<commit_message>
feat(chart): Phase 2 — Bollinger Bands, VWAP, custom-period SMA on price pane
- BB (20,2): BollingerSeries + BollingerBandTooltip; price-pane y-extents
  expanded to include band top/bottom so lines never clip.
- VWAP: anchored cumulative typical-price × volume, rendered as LineSeries.
- SMA: user-configurable windowSize (default 20, clamped 2–200) with
  number input embedded in the indicator dropdown row.
- INDICATOR_OPTIONS extended with bb / vwap / sma (default off to avoid
  clutter on first load).
- ROADMAP: Phase 2 + C-201…C-204 marked Done; Session Log appended with
  handoff to Phase 3 (Stochastic, ATR, paneConfig refactor).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/roadmap_version_2.xlsx
+++ b/stockpredict/roadmap_version_2.xlsx
@@ -197,7 +197,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -289,6 +289,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -768,7 +771,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Overlay Indicators</t>
+          <t>Overlay Indicators ✅</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -792,12 +795,12 @@
       </c>
       <c r="F6" s="11" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>All use LineSeries / BollingerSeries — same pane, same price scale. No new pane needed.</t>
+          <t>Completed 2026-05-25. BB, VWAP, custom-period SMA — all on price pane.</t>
         </is>
       </c>
     </row>
@@ -1300,7 +1303,7 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2 ✅</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -1325,7 +1328,7 @@
       </c>
       <c r="G9" s="11" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr"/>
@@ -1343,7 +1346,7 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2 ✅</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -1368,7 +1371,7 @@
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr"/>
@@ -1386,7 +1389,7 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2 ✅</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -1411,7 +1414,7 @@
       </c>
       <c r="G11" s="11" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr"/>
@@ -1429,7 +1432,7 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2 ✅</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -1454,7 +1457,7 @@
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
@@ -2067,7 +2070,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2208,6 +2211,49 @@
       <c r="D10" s="29" t="inlineStr"/>
       <c r="E10" s="29" t="inlineStr"/>
       <c r="F10" s="29" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B11" s="33" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="C11" s="33" t="inlineStr">
+        <is>
+          <t>C-201 Bollinger Bands (20,2)
+C-202 VWAP (anchored cumulative)
+C-203 Custom-period SMA + number input
+C-204 Extended INDICATOR_OPTIONS</t>
+        </is>
+      </c>
+      <c r="D11" s="33" t="inlineStr">
+        <is>
+          <t>StockChart.js
+roadmap_version_2.xlsx</t>
+        </is>
+      </c>
+      <c r="E11" s="33" t="inlineStr">
+        <is>
+          <t>Phase 2 done. Production build clean (only pre-existing
+ESLint warnings in unrelated files).
+New indicators default OFF to avoid initial clutter.
+BB tooltip at origin [8,40]; SMA period input in dropdown
+(clamped 2–200).</t>
+        </is>
+      </c>
+      <c r="F11" s="33" t="inlineStr">
+        <is>
+          <t>Phase 3: Stochastic Oscillator pane (C-301), ATR pane (C-302),
+paneConfig refactor (C-303).
+Tip: refactor hardcoded pane heights into a paneConfig[] array
+first — Phase 3 introduces 2 new panes.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
feat(chart): Phase 3 — Stochastic + ATR panes, paneConfig refactor
- paneConfig refactor (C-303): replace hardcoded macdHeight/volHeight with
  SUB_PANE_HEIGHTS={macd,stoch,atr,volume} + computed paneOrigin lookup.
  Bottom-most enabled sub-pane now owns the date tick labels and
  MouseCoordinateX (previously hard-pinned to volume).
- Stochastic Oscillator (C-301): new pane id=5, stochasticOscillator(12,3,3),
  StochasticSeries with reference lines at 20/80, StochasticTooltip.
- ATR (C-302): new pane id=6, atr(14) → LineSeries (cyan) with
  SingleValueTooltip; auto y-extents.
- Both new indicators default OFF.
- ROADMAP: Phase 3 + C-301..C-303 marked Done; Session Log appended with
  handoff to Phase 4 (drawing tools).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/roadmap_version_2.xlsx
+++ b/stockpredict/roadmap_version_2.xlsx
@@ -812,7 +812,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>More Oscillators</t>
+          <t>More Oscillators ✅</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -835,12 +835,12 @@
       </c>
       <c r="F7" s="11" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>react-financial-charts has stochasticOscillator() and atr() calculators + series.</t>
+          <t>Completed 2026-05-25. Stochastic (12,3,3) and ATR (14) panes; paneConfig refactor — sub-pane origins computed from SUB_PANE_HEIGHTS + enabled flags. Bottom-most enabled sub-pane shows date tick labels.</t>
         </is>
       </c>
     </row>
@@ -1479,7 +1479,7 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>3 ✅</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="G13" s="11" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr"/>
@@ -1522,7 +1522,7 @@
       </c>
       <c r="B14" s="12" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>3 ✅</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -1547,7 +1547,7 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr"/>
@@ -1565,7 +1565,7 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>3 ✅</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -1590,7 +1590,7 @@
       </c>
       <c r="G15" s="11" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
@@ -2070,7 +2070,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2252,6 +2252,50 @@
 paneConfig refactor (C-303).
 Tip: refactor hardcoded pane heights into a paneConfig[] array
 first — Phase 3 introduces 2 new panes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B12" s="33" t="inlineStr">
+        <is>
+          <t>Phase 3</t>
+        </is>
+      </c>
+      <c r="C12" s="33" t="inlineStr">
+        <is>
+          <t>C-303 paneConfig refactor (SUB_PANE_HEIGHTS + paneOrigin lookup)
+C-301 Stochastic Oscillator pane (12,3,3) with %K/%D + tooltip
+C-302 ATR (14) pane — LineSeries + SingleValueTooltip</t>
+        </is>
+      </c>
+      <c r="D12" s="33" t="inlineStr">
+        <is>
+          <t>StockChart.js
+roadmap_version_2.xlsx</t>
+        </is>
+      </c>
+      <c r="E12" s="33" t="inlineStr">
+        <is>
+          <t>Phase 3 done. Same session as Phase 2.
+Refactor first: hardcoded macdHeight/volHeight replaced with
+SUB_PANE_HEIGHTS={macd,stoch,atr,volume} and computed paneOrigin.
+Bottom-most enabled sub-pane now owns the date tick labels +
+MouseCoordinateX (previously only volume showed them).
+Stochastic and ATR default OFF.
+Production build clean (+771 B gzipped).</t>
+        </is>
+      </c>
+      <c r="F12" s="33" t="inlineStr">
+        <is>
+          <t>Phase 4: Drawing tools — trend line (C-401), horizontal S/R (C-402),
+Fibonacci (C-403), drawing toolbar UI (C-404).
+Requires @react-financial-charts/interactive (already bundled in v2).
+New DrawingToolbar.js component + persisted drawings array state.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor(chart): remove legacy bootstrap buttons + stub Select from CompanyCharts
Now redundant after Phase 5 added internal timeframe tabs inside
StockChart. Drops:

- 1w/1m/1y/5y/All bootstrap ButtonGroup + click handlers
- stub react-dropdown-select listing "Leanne Graham"/"Ervin Howell"
- periodStockData slicing state (StockChart now slices internally)
- inline bootstrap.min.css import (only this file imported it as a
  relative node_modules path; other consumers go through the bare
  specifier, so the bundle drops ~18 KB gzipped)
- unused selectItem/styles/options + debug console.log

CompanyCharts is now just: fetch history → loading guard → render
StockChart with the symbol prop. -105 / +26 lines.

react-bootstrap stays in package.json — Solutions/TimeSeries/Agent
pages still use it.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/roadmap_version_2.xlsx
+++ b/stockpredict/roadmap_version_2.xlsx
@@ -2070,7 +2070,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2400,6 +2400,53 @@
   • Remove the legacy bootstrap buttons in CompanyCharts (now
     redundant with the internal timeframe tabs)
   • Clean up stub Select for "Leanne Graham" / "Ervin Howell"</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B15" s="33" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C15" s="33" t="inlineStr">
+        <is>
+          <t>Removed legacy bootstrap buttons (1w/1m/1y/5y/All) + stub
+react-dropdown-select ("Leanne Graham") from CompanyCharts.js.
+Now redundant after Phase 5 internal timeframe tabs in StockChart.
+Also dropped: periodStockData slicing state, debug console.log,
+unused selectItem/styles/options.</t>
+        </is>
+      </c>
+      <c r="D15" s="33" t="inlineStr">
+        <is>
+          <t>CompanyCharts.js</t>
+        </is>
+      </c>
+      <c r="E15" s="33" t="inlineStr">
+        <is>
+          <t>Browser-verified Phases 2–5 working end-to-end on port 3004
+(user signed off: "beautiful charts").
+Cleanup: −105 / +26 lines in CompanyCharts.js.
+Bundle: −18 kB gzipped (vs. Phase 4 commit) — bootstrap CSS
+was being imported via this file. react-bootstrap stays as a
+dependency since Solutions/TimeSeries/Agent pages still use it.</t>
+        </is>
+      </c>
+      <c r="F15" s="33" t="inlineStr">
+        <is>
+          <t>Polish backlog remaining:
+  • DrawingObjectSelector + DEL key for per-item drawing delete
+  • Snap-to-bar option for trend lines (snap={true}+snapTo)
+  • Misleading "demo / password" hint on login screen (server
+    rejects with 422 — email field validated as email)
+  • Transient &lt;rect&gt; negative-height SVG warning at chart init
+  • Phase 6 (multi-stock compare) — XL, still Not Started</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(auth): drop misleading "demo / password" hint on login screen
The hint advertised `demo` / `password`, but the auth-service
validates the username field as an email and rejects `demo` with
HTTP 422 — no demo user is seeded. Removed:

- The JSX block in LoginForm.js (auth-demo / auth-demo-text).
- The matching CSS rules in auth.css.
- The login.demo_account translation keys in en.json and vi.json.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/roadmap_version_2.xlsx
+++ b/stockpredict/roadmap_version_2.xlsx
@@ -2070,7 +2070,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2447,6 +2447,48 @@
     rejects with 422 — email field validated as email)
   • Transient &lt;rect&gt; negative-height SVG warning at chart init
   • Phase 6 (multi-stock compare) — XL, still Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B16" s="33" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C16" s="33" t="inlineStr">
+        <is>
+          <t>Removed misleading "Demo account: demo/password" hint from LoginForm.</t>
+        </is>
+      </c>
+      <c r="D16" s="33" t="inlineStr">
+        <is>
+          <t>LoginForm.js
+auth.css
+en.json / vi.json</t>
+        </is>
+      </c>
+      <c r="E16" s="33" t="inlineStr">
+        <is>
+          <t>Hint was broken: auth-service validates the username field as an
+email and rejected "demo" with 422. No demo user was seeded.
+Removed JSX block, .auth-demo / .auth-demo-text CSS rules, and
+login.demo_account translation keys in both locales.
+Bundle: −92 B gzipped (JS), −41 B (CSS).</t>
+        </is>
+      </c>
+      <c r="F16" s="33" t="inlineStr">
+        <is>
+          <t>Polish backlog still open:
+  • DrawingObjectSelector + DEL key for per-item drawing delete
+  • Snap-to-bar for trend lines
+  • Transient &lt;rect&gt; negative-height SVG warning at chart init
+  • Phase 6 (multi-stock compare)</t>
         </is>
       </c>
     </row>

</xml_diff>